<commit_message>
Add boarders for free text.
</commit_message>
<xml_diff>
--- a/technique_overlay_inputs.xlsx
+++ b/technique_overlay_inputs.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rhys.r.evans/Documents/CEDA/CCI/cci_data_bridge_inputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A855E59-440E-7B4A-B63A-B4B7CE932B38}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE342CE2-25C7-FA4F-BC37-E310A72C17D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="38400" windowHeight="19320" xr2:uid="{1975E336-1F0E-40CF-A2E0-F60BE7832FDC}"/>
   </bookViews>
@@ -567,7 +567,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="12">
+  <borders count="13">
     <border>
       <left/>
       <right/>
@@ -690,12 +690,25 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -725,9 +738,6 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -778,6 +788,16 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1130,24 +1150,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A1" s="20" t="s">
+      <c r="A1" s="19" t="s">
         <v>33</v>
       </c>
-      <c r="B1" s="20"/>
-      <c r="C1" s="21"/>
-      <c r="D1" s="18" t="s">
+      <c r="B1" s="19"/>
+      <c r="C1" s="20"/>
+      <c r="D1" s="17" t="s">
         <v>34</v>
       </c>
-      <c r="E1" s="22" t="s">
+      <c r="E1" s="21" t="s">
         <v>35</v>
       </c>
-      <c r="F1" s="24" t="s">
+      <c r="F1" s="23" t="s">
         <v>36</v>
       </c>
-      <c r="G1" s="20"/>
-      <c r="H1" s="20"/>
-      <c r="I1" s="25"/>
-      <c r="J1" s="26" t="s">
+      <c r="G1" s="19"/>
+      <c r="H1" s="19"/>
+      <c r="I1" s="24"/>
+      <c r="J1" s="25" t="s">
         <v>37</v>
       </c>
     </row>
@@ -1161,8 +1181,8 @@
       <c r="C2" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="D2" s="19"/>
-      <c r="E2" s="23"/>
+      <c r="D2" s="18"/>
+      <c r="E2" s="22"/>
       <c r="F2" s="2" t="s">
         <v>40</v>
       </c>
@@ -1175,7 +1195,7 @@
       <c r="I2" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="J2" s="27"/>
+      <c r="J2" s="26"/>
     </row>
     <row r="3" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A3" s="5" t="s">
@@ -1205,7 +1225,7 @@
       <c r="I3" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="J3" s="3" t="s">
+      <c r="J3" s="28" t="s">
         <v>50</v>
       </c>
     </row>
@@ -1237,7 +1257,7 @@
       <c r="I4" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="J4" s="3" t="s">
+      <c r="J4" s="29" t="s">
         <v>48</v>
       </c>
     </row>
@@ -1269,7 +1289,7 @@
       <c r="I5" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="J5" s="3" t="s">
+      <c r="J5" s="29" t="s">
         <v>29</v>
       </c>
     </row>
@@ -1301,7 +1321,7 @@
       <c r="I6" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="J6" s="3" t="s">
+      <c r="J6" s="29" t="s">
         <v>31</v>
       </c>
     </row>
@@ -1333,7 +1353,7 @@
       <c r="I7" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="J7" s="3" t="s">
+      <c r="J7" s="29" t="s">
         <v>29</v>
       </c>
     </row>
@@ -1365,7 +1385,7 @@
       <c r="I8" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="J8" s="3" t="s">
+      <c r="J8" s="29" t="s">
         <v>31</v>
       </c>
     </row>
@@ -1397,7 +1417,7 @@
       <c r="I9" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="J9" s="3" t="s">
+      <c r="J9" s="29" t="s">
         <v>32</v>
       </c>
     </row>
@@ -1426,15 +1446,15 @@
       <c r="H10" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="I10" s="11" t="s">
+      <c r="I10" s="27" t="s">
         <v>6</v>
       </c>
-      <c r="J10" s="12" t="s">
+      <c r="J10" s="11" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="11" spans="1:10" ht="16" x14ac:dyDescent="0.2">
-      <c r="A11" s="13" t="s">
+      <c r="A11" s="12" t="s">
         <v>44</v>
       </c>
       <c r="B11" s="8" t="s">
@@ -1458,21 +1478,21 @@
       <c r="H11" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="I11" s="11" t="s">
+      <c r="I11" s="27" t="s">
         <v>8</v>
       </c>
-      <c r="J11" s="12" t="s">
+      <c r="J11" s="11" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="12" spans="1:10" ht="16" x14ac:dyDescent="0.2">
-      <c r="A12" s="13" t="s">
+      <c r="A12" s="12" t="s">
         <v>44</v>
       </c>
       <c r="B12" s="8" t="s">
         <v>53</v>
       </c>
-      <c r="C12" s="16" t="s">
+      <c r="C12" s="15" t="s">
         <v>52</v>
       </c>
       <c r="D12" s="6" t="s">
@@ -1493,18 +1513,18 @@
       <c r="I12" t="s">
         <v>20</v>
       </c>
-      <c r="J12" t="s">
+      <c r="J12" s="30" t="s">
         <v>54</v>
       </c>
     </row>
     <row r="13" spans="1:10" ht="16" x14ac:dyDescent="0.2">
-      <c r="A13" s="13" t="s">
+      <c r="A13" s="12" t="s">
         <v>44</v>
       </c>
       <c r="B13" s="8" t="s">
         <v>53</v>
       </c>
-      <c r="C13" s="16" t="s">
+      <c r="C13" s="15" t="s">
         <v>23</v>
       </c>
       <c r="D13" s="6" t="s">
@@ -1525,18 +1545,18 @@
       <c r="I13" t="s">
         <v>14</v>
       </c>
-      <c r="J13" t="s">
+      <c r="J13" s="30" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="14" spans="1:10" ht="16" x14ac:dyDescent="0.2">
-      <c r="A14" s="13" t="s">
+      <c r="A14" s="12" t="s">
         <v>44</v>
       </c>
       <c r="B14" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="C14" s="14" t="s">
+      <c r="C14" s="13" t="s">
         <v>11</v>
       </c>
       <c r="D14" s="6" t="s">
@@ -1554,21 +1574,21 @@
       <c r="H14" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="I14" s="11" t="s">
+      <c r="I14" s="27" t="s">
         <v>12</v>
       </c>
-      <c r="J14" s="12" t="s">
+      <c r="J14" s="11" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="15" spans="1:10" ht="16" x14ac:dyDescent="0.2">
-      <c r="A15" s="13" t="s">
+      <c r="A15" s="12" t="s">
         <v>44</v>
       </c>
       <c r="B15" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="C15" s="14" t="s">
+      <c r="C15" s="13" t="s">
         <v>11</v>
       </c>
       <c r="D15" s="6" t="s">
@@ -1586,21 +1606,21 @@
       <c r="H15" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="I15" s="11" t="s">
+      <c r="I15" s="27" t="s">
         <v>14</v>
       </c>
-      <c r="J15" s="12" t="s">
+      <c r="J15" s="11" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="16" spans="1:10" ht="16" x14ac:dyDescent="0.2">
-      <c r="A16" s="13" t="s">
+      <c r="A16" s="12" t="s">
         <v>44</v>
       </c>
       <c r="B16" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="C16" s="17" t="s">
+      <c r="C16" s="16" t="s">
         <v>23</v>
       </c>
       <c r="D16" s="6" t="s">
@@ -1621,18 +1641,18 @@
       <c r="I16" t="s">
         <v>14</v>
       </c>
-      <c r="J16" t="s">
+      <c r="J16" s="30" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="17" spans="1:11" ht="16" x14ac:dyDescent="0.2">
-      <c r="A17" s="13" t="s">
+      <c r="A17" s="12" t="s">
         <v>44</v>
       </c>
       <c r="B17" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="C17" s="17" t="s">
+      <c r="C17" s="16" t="s">
         <v>23</v>
       </c>
       <c r="D17" s="6" t="s">
@@ -1653,18 +1673,18 @@
       <c r="I17" t="s">
         <v>12</v>
       </c>
-      <c r="J17" t="s">
+      <c r="J17" s="30" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="18" spans="1:11" ht="16" x14ac:dyDescent="0.2">
-      <c r="A18" s="13" t="s">
+      <c r="A18" s="12" t="s">
         <v>44</v>
       </c>
       <c r="B18" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="C18" s="17" t="s">
+      <c r="C18" s="16" t="s">
         <v>23</v>
       </c>
       <c r="D18" s="6" t="s">
@@ -1685,18 +1705,18 @@
       <c r="I18" t="s">
         <v>8</v>
       </c>
-      <c r="J18" t="s">
+      <c r="J18" s="30" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="19" spans="1:11" ht="16" x14ac:dyDescent="0.2">
-      <c r="A19" s="13" t="s">
+      <c r="A19" s="12" t="s">
         <v>44</v>
       </c>
       <c r="B19" t="s">
         <v>60</v>
       </c>
-      <c r="C19" s="17" t="s">
+      <c r="C19" s="16" t="s">
         <v>23</v>
       </c>
       <c r="D19" s="6" t="s">
@@ -1717,19 +1737,19 @@
       <c r="I19" t="s">
         <v>20</v>
       </c>
-      <c r="J19" t="s">
+      <c r="J19" s="30" t="s">
         <v>61</v>
       </c>
       <c r="K19"/>
     </row>
     <row r="20" spans="1:11" ht="16" x14ac:dyDescent="0.2">
-      <c r="A20" s="13" t="s">
+      <c r="A20" s="12" t="s">
         <v>44</v>
       </c>
       <c r="B20" t="s">
         <v>60</v>
       </c>
-      <c r="C20" s="17" t="s">
+      <c r="C20" s="16" t="s">
         <v>23</v>
       </c>
       <c r="D20" s="6" t="s">
@@ -1750,19 +1770,19 @@
       <c r="I20" t="s">
         <v>8</v>
       </c>
-      <c r="J20" t="s">
+      <c r="J20" s="30" t="s">
         <v>62</v>
       </c>
       <c r="K20"/>
     </row>
     <row r="21" spans="1:11" ht="16" x14ac:dyDescent="0.2">
-      <c r="A21" s="13" t="s">
+      <c r="A21" s="12" t="s">
         <v>44</v>
       </c>
       <c r="B21" t="s">
         <v>60</v>
       </c>
-      <c r="C21" s="17" t="s">
+      <c r="C21" s="16" t="s">
         <v>23</v>
       </c>
       <c r="D21" s="6" t="s">
@@ -1783,19 +1803,19 @@
       <c r="I21" t="s">
         <v>8</v>
       </c>
-      <c r="J21" t="s">
+      <c r="J21" s="30" t="s">
         <v>64</v>
       </c>
       <c r="K21"/>
     </row>
     <row r="22" spans="1:11" ht="16" x14ac:dyDescent="0.2">
-      <c r="A22" s="13" t="s">
+      <c r="A22" s="12" t="s">
         <v>44</v>
       </c>
       <c r="B22" t="s">
         <v>65</v>
       </c>
-      <c r="C22" s="17" t="s">
+      <c r="C22" s="16" t="s">
         <v>23</v>
       </c>
       <c r="D22" s="6" t="s">
@@ -1816,19 +1836,19 @@
       <c r="I22" t="s">
         <v>20</v>
       </c>
-      <c r="J22" t="s">
+      <c r="J22" s="30" t="s">
         <v>67</v>
       </c>
       <c r="K22"/>
     </row>
     <row r="23" spans="1:11" ht="16" x14ac:dyDescent="0.2">
-      <c r="A23" s="13" t="s">
+      <c r="A23" s="12" t="s">
         <v>44</v>
       </c>
       <c r="B23" t="s">
         <v>65</v>
       </c>
-      <c r="C23" s="17" t="s">
+      <c r="C23" s="16" t="s">
         <v>23</v>
       </c>
       <c r="D23" s="6" t="s">
@@ -1849,19 +1869,19 @@
       <c r="I23" t="s">
         <v>20</v>
       </c>
-      <c r="J23" t="s">
+      <c r="J23" s="30" t="s">
         <v>69</v>
       </c>
       <c r="K23"/>
     </row>
     <row r="24" spans="1:11" ht="16" x14ac:dyDescent="0.2">
-      <c r="A24" s="13" t="s">
+      <c r="A24" s="12" t="s">
         <v>44</v>
       </c>
       <c r="B24" t="s">
         <v>65</v>
       </c>
-      <c r="C24" s="17" t="s">
+      <c r="C24" s="16" t="s">
         <v>23</v>
       </c>
       <c r="D24" s="6" t="s">
@@ -1882,19 +1902,19 @@
       <c r="I24" t="s">
         <v>12</v>
       </c>
-      <c r="J24" t="s">
+      <c r="J24" s="30" t="s">
         <v>72</v>
       </c>
       <c r="K24"/>
     </row>
     <row r="25" spans="1:11" ht="16" x14ac:dyDescent="0.2">
-      <c r="A25" s="13" t="s">
+      <c r="A25" s="12" t="s">
         <v>44</v>
       </c>
       <c r="B25" t="s">
         <v>65</v>
       </c>
-      <c r="C25" s="17" t="s">
+      <c r="C25" s="16" t="s">
         <v>23</v>
       </c>
       <c r="D25" s="6" t="s">
@@ -1915,19 +1935,19 @@
       <c r="I25" t="s">
         <v>14</v>
       </c>
-      <c r="J25" t="s">
+      <c r="J25" s="30" t="s">
         <v>75</v>
       </c>
       <c r="K25"/>
     </row>
     <row r="26" spans="1:11" ht="16" x14ac:dyDescent="0.2">
-      <c r="A26" s="13" t="s">
+      <c r="A26" s="12" t="s">
         <v>44</v>
       </c>
       <c r="B26" t="s">
         <v>65</v>
       </c>
-      <c r="C26" s="17" t="s">
+      <c r="C26" s="16" t="s">
         <v>23</v>
       </c>
       <c r="D26" s="6" t="s">
@@ -1948,19 +1968,19 @@
       <c r="I26" t="s">
         <v>14</v>
       </c>
-      <c r="J26" t="s">
+      <c r="J26" s="30" t="s">
         <v>77</v>
       </c>
       <c r="K26"/>
     </row>
     <row r="27" spans="1:11" ht="16" x14ac:dyDescent="0.2">
-      <c r="A27" s="13" t="s">
+      <c r="A27" s="12" t="s">
         <v>44</v>
       </c>
       <c r="B27" t="s">
         <v>78</v>
       </c>
-      <c r="C27" s="17" t="s">
+      <c r="C27" s="16" t="s">
         <v>23</v>
       </c>
       <c r="D27" s="6" t="s">
@@ -1981,19 +2001,19 @@
       <c r="I27" t="s">
         <v>14</v>
       </c>
-      <c r="J27" t="s">
+      <c r="J27" s="30" t="s">
         <v>80</v>
       </c>
       <c r="K27"/>
     </row>
     <row r="28" spans="1:11" ht="16" x14ac:dyDescent="0.2">
-      <c r="A28" s="13" t="s">
+      <c r="A28" s="12" t="s">
         <v>44</v>
       </c>
       <c r="B28" t="s">
         <v>78</v>
       </c>
-      <c r="C28" s="17" t="s">
+      <c r="C28" s="16" t="s">
         <v>23</v>
       </c>
       <c r="D28" s="6" t="s">
@@ -2014,19 +2034,19 @@
       <c r="I28" t="s">
         <v>14</v>
       </c>
-      <c r="J28" t="s">
+      <c r="J28" s="30" t="s">
         <v>82</v>
       </c>
       <c r="K28"/>
     </row>
     <row r="29" spans="1:11" ht="16" x14ac:dyDescent="0.2">
-      <c r="A29" s="13" t="s">
+      <c r="A29" s="12" t="s">
         <v>44</v>
       </c>
       <c r="B29" t="s">
         <v>78</v>
       </c>
-      <c r="C29" s="17" t="s">
+      <c r="C29" s="16" t="s">
         <v>23</v>
       </c>
       <c r="D29" s="6" t="s">
@@ -2047,19 +2067,19 @@
       <c r="I29" t="s">
         <v>12</v>
       </c>
-      <c r="J29" t="s">
+      <c r="J29" s="30" t="s">
         <v>83</v>
       </c>
       <c r="K29"/>
     </row>
     <row r="30" spans="1:11" ht="16" x14ac:dyDescent="0.2">
-      <c r="A30" s="13" t="s">
+      <c r="A30" s="12" t="s">
         <v>44</v>
       </c>
       <c r="B30" t="s">
         <v>84</v>
       </c>
-      <c r="C30" s="17" t="s">
+      <c r="C30" s="16" t="s">
         <v>23</v>
       </c>
       <c r="D30" s="6" t="s">
@@ -2080,19 +2100,19 @@
       <c r="I30" t="s">
         <v>14</v>
       </c>
-      <c r="J30" t="s">
+      <c r="J30" s="30" t="s">
         <v>85</v>
       </c>
       <c r="K30"/>
     </row>
     <row r="31" spans="1:11" ht="16" x14ac:dyDescent="0.2">
-      <c r="A31" s="13" t="s">
+      <c r="A31" s="12" t="s">
         <v>44</v>
       </c>
       <c r="B31" t="s">
         <v>84</v>
       </c>
-      <c r="C31" s="17" t="s">
+      <c r="C31" s="16" t="s">
         <v>23</v>
       </c>
       <c r="D31" s="6" t="s">
@@ -2113,19 +2133,19 @@
       <c r="I31" t="s">
         <v>12</v>
       </c>
-      <c r="J31" t="s">
+      <c r="J31" s="30" t="s">
         <v>86</v>
       </c>
       <c r="K31"/>
     </row>
     <row r="32" spans="1:11" ht="16" x14ac:dyDescent="0.2">
-      <c r="A32" s="13" t="s">
+      <c r="A32" s="12" t="s">
         <v>44</v>
       </c>
       <c r="B32" t="s">
         <v>87</v>
       </c>
-      <c r="C32" s="17" t="s">
+      <c r="C32" s="16" t="s">
         <v>23</v>
       </c>
       <c r="D32" s="6" t="s">
@@ -2146,19 +2166,19 @@
       <c r="I32" t="s">
         <v>89</v>
       </c>
-      <c r="J32" t="s">
+      <c r="J32" s="30" t="s">
         <v>90</v>
       </c>
       <c r="K32"/>
     </row>
     <row r="33" spans="1:11" ht="16" x14ac:dyDescent="0.2">
-      <c r="A33" s="13" t="s">
+      <c r="A33" s="12" t="s">
         <v>44</v>
       </c>
       <c r="B33" t="s">
         <v>87</v>
       </c>
-      <c r="C33" s="17" t="s">
+      <c r="C33" s="16" t="s">
         <v>23</v>
       </c>
       <c r="D33" s="6" t="s">
@@ -2179,19 +2199,19 @@
       <c r="I33" t="s">
         <v>20</v>
       </c>
-      <c r="J33" t="s">
+      <c r="J33" s="30" t="s">
         <v>92</v>
       </c>
       <c r="K33"/>
     </row>
     <row r="34" spans="1:11" ht="16" x14ac:dyDescent="0.2">
-      <c r="A34" s="13" t="s">
+      <c r="A34" s="12" t="s">
         <v>44</v>
       </c>
       <c r="B34" t="s">
         <v>87</v>
       </c>
-      <c r="C34" s="17" t="s">
+      <c r="C34" s="16" t="s">
         <v>23</v>
       </c>
       <c r="D34" s="6" t="s">
@@ -2212,19 +2232,19 @@
       <c r="I34" t="s">
         <v>20</v>
       </c>
-      <c r="J34" t="s">
+      <c r="J34" s="30" t="s">
         <v>93</v>
       </c>
       <c r="K34"/>
     </row>
     <row r="35" spans="1:11" ht="16" x14ac:dyDescent="0.2">
-      <c r="A35" s="13" t="s">
+      <c r="A35" s="12" t="s">
         <v>44</v>
       </c>
       <c r="B35" t="s">
         <v>94</v>
       </c>
-      <c r="C35" s="17" t="s">
+      <c r="C35" s="16" t="s">
         <v>23</v>
       </c>
       <c r="D35" s="6" t="s">
@@ -2245,18 +2265,18 @@
       <c r="I35" t="s">
         <v>95</v>
       </c>
-      <c r="J35" t="s">
+      <c r="J35" s="30" t="s">
         <v>96</v>
       </c>
     </row>
     <row r="36" spans="1:11" ht="16" x14ac:dyDescent="0.2">
-      <c r="A36" s="13" t="s">
+      <c r="A36" s="12" t="s">
         <v>44</v>
       </c>
       <c r="B36" t="s">
         <v>94</v>
       </c>
-      <c r="C36" s="17" t="s">
+      <c r="C36" s="16" t="s">
         <v>23</v>
       </c>
       <c r="D36" s="6" t="s">
@@ -2277,18 +2297,18 @@
       <c r="I36" t="s">
         <v>8</v>
       </c>
-      <c r="J36" t="s">
+      <c r="J36" s="30" t="s">
         <v>97</v>
       </c>
     </row>
     <row r="37" spans="1:11" ht="16" x14ac:dyDescent="0.2">
-      <c r="A37" s="13" t="s">
+      <c r="A37" s="12" t="s">
         <v>44</v>
       </c>
       <c r="B37" t="s">
         <v>94</v>
       </c>
-      <c r="C37" s="17" t="s">
+      <c r="C37" s="16" t="s">
         <v>23</v>
       </c>
       <c r="D37" s="6" t="s">
@@ -2309,18 +2329,18 @@
       <c r="I37" t="s">
         <v>95</v>
       </c>
-      <c r="J37" t="s">
+      <c r="J37" s="30" t="s">
         <v>96</v>
       </c>
     </row>
     <row r="38" spans="1:11" ht="16" x14ac:dyDescent="0.2">
-      <c r="A38" s="13" t="s">
+      <c r="A38" s="12" t="s">
         <v>44</v>
       </c>
       <c r="B38" t="s">
         <v>94</v>
       </c>
-      <c r="C38" s="17" t="s">
+      <c r="C38" s="16" t="s">
         <v>23</v>
       </c>
       <c r="D38" s="6" t="s">
@@ -2341,18 +2361,18 @@
       <c r="I38" t="s">
         <v>8</v>
       </c>
-      <c r="J38" t="s">
+      <c r="J38" s="30" t="s">
         <v>97</v>
       </c>
     </row>
     <row r="39" spans="1:11" ht="16" x14ac:dyDescent="0.2">
-      <c r="A39" s="13" t="s">
+      <c r="A39" s="12" t="s">
         <v>44</v>
       </c>
       <c r="B39" t="s">
         <v>94</v>
       </c>
-      <c r="C39" s="17" t="s">
+      <c r="C39" s="16" t="s">
         <v>23</v>
       </c>
       <c r="D39" s="6" t="s">
@@ -2373,18 +2393,18 @@
       <c r="I39" t="s">
         <v>20</v>
       </c>
-      <c r="J39" t="s">
+      <c r="J39" s="30" t="s">
         <v>99</v>
       </c>
     </row>
     <row r="40" spans="1:11" ht="16" x14ac:dyDescent="0.2">
-      <c r="A40" s="13" t="s">
+      <c r="A40" s="12" t="s">
         <v>44</v>
       </c>
       <c r="B40" t="s">
         <v>94</v>
       </c>
-      <c r="C40" s="17" t="s">
+      <c r="C40" s="16" t="s">
         <v>23</v>
       </c>
       <c r="D40" s="6" t="s">
@@ -2405,18 +2425,18 @@
       <c r="I40" t="s">
         <v>6</v>
       </c>
-      <c r="J40" t="s">
+      <c r="J40" s="30" t="s">
         <v>101</v>
       </c>
     </row>
     <row r="41" spans="1:11" ht="16" x14ac:dyDescent="0.2">
-      <c r="A41" s="13" t="s">
+      <c r="A41" s="12" t="s">
         <v>44</v>
       </c>
       <c r="B41" t="s">
         <v>94</v>
       </c>
-      <c r="C41" s="17" t="s">
+      <c r="C41" s="16" t="s">
         <v>23</v>
       </c>
       <c r="D41" s="6" t="s">
@@ -2437,18 +2457,18 @@
       <c r="I41" t="s">
         <v>14</v>
       </c>
-      <c r="J41" t="s">
+      <c r="J41" s="30" t="s">
         <v>102</v>
       </c>
     </row>
     <row r="42" spans="1:11" ht="16" x14ac:dyDescent="0.2">
-      <c r="A42" s="13" t="s">
+      <c r="A42" s="12" t="s">
         <v>44</v>
       </c>
       <c r="B42" t="s">
         <v>94</v>
       </c>
-      <c r="C42" s="17" t="s">
+      <c r="C42" s="16" t="s">
         <v>23</v>
       </c>
       <c r="D42" s="6" t="s">
@@ -2469,18 +2489,18 @@
       <c r="I42" t="s">
         <v>14</v>
       </c>
-      <c r="J42" t="s">
+      <c r="J42" s="30" t="s">
         <v>102</v>
       </c>
     </row>
     <row r="43" spans="1:11" ht="16" x14ac:dyDescent="0.2">
-      <c r="A43" s="13" t="s">
+      <c r="A43" s="12" t="s">
         <v>44</v>
       </c>
       <c r="B43" t="s">
         <v>103</v>
       </c>
-      <c r="C43" s="17" t="s">
+      <c r="C43" s="16" t="s">
         <v>23</v>
       </c>
       <c r="D43" s="6" t="s">
@@ -2501,18 +2521,18 @@
       <c r="I43" t="s">
         <v>14</v>
       </c>
-      <c r="J43" t="s">
+      <c r="J43" s="30" t="s">
         <v>104</v>
       </c>
     </row>
     <row r="44" spans="1:11" ht="16" x14ac:dyDescent="0.2">
-      <c r="A44" s="13" t="s">
+      <c r="A44" s="12" t="s">
         <v>44</v>
       </c>
       <c r="B44" t="s">
         <v>103</v>
       </c>
-      <c r="C44" s="17" t="s">
+      <c r="C44" s="16" t="s">
         <v>23</v>
       </c>
       <c r="D44" s="6" t="s">
@@ -2533,18 +2553,18 @@
       <c r="I44" t="s">
         <v>14</v>
       </c>
-      <c r="J44" t="s">
+      <c r="J44" s="30" t="s">
         <v>105</v>
       </c>
     </row>
     <row r="45" spans="1:11" ht="16" x14ac:dyDescent="0.2">
-      <c r="A45" s="13" t="s">
+      <c r="A45" s="12" t="s">
         <v>44</v>
       </c>
       <c r="B45" t="s">
         <v>103</v>
       </c>
-      <c r="C45" s="17" t="s">
+      <c r="C45" s="16" t="s">
         <v>23</v>
       </c>
       <c r="D45" s="6" t="s">
@@ -2565,18 +2585,18 @@
       <c r="I45" t="s">
         <v>8</v>
       </c>
-      <c r="J45" t="s">
+      <c r="J45" s="30" t="s">
         <v>106</v>
       </c>
     </row>
     <row r="46" spans="1:11" ht="16" x14ac:dyDescent="0.2">
-      <c r="A46" s="13" t="s">
+      <c r="A46" s="12" t="s">
         <v>44</v>
       </c>
       <c r="B46" t="s">
         <v>103</v>
       </c>
-      <c r="C46" s="17" t="s">
+      <c r="C46" s="16" t="s">
         <v>23</v>
       </c>
       <c r="D46" s="6" t="s">
@@ -2597,18 +2617,18 @@
       <c r="I46" t="s">
         <v>8</v>
       </c>
-      <c r="J46" t="s">
+      <c r="J46" s="30" t="s">
         <v>107</v>
       </c>
     </row>
     <row r="47" spans="1:11" ht="16" x14ac:dyDescent="0.2">
-      <c r="A47" s="13" t="s">
+      <c r="A47" s="12" t="s">
         <v>44</v>
       </c>
       <c r="B47" t="s">
         <v>103</v>
       </c>
-      <c r="C47" s="17" t="s">
+      <c r="C47" s="16" t="s">
         <v>23</v>
       </c>
       <c r="D47" s="6" t="s">
@@ -2629,18 +2649,18 @@
       <c r="I47" t="s">
         <v>95</v>
       </c>
-      <c r="J47" t="s">
+      <c r="J47" s="30" t="s">
         <v>108</v>
       </c>
     </row>
     <row r="48" spans="1:11" ht="16" x14ac:dyDescent="0.2">
-      <c r="A48" s="13" t="s">
+      <c r="A48" s="12" t="s">
         <v>44</v>
       </c>
       <c r="B48" t="s">
         <v>109</v>
       </c>
-      <c r="C48" s="17" t="s">
+      <c r="C48" s="16" t="s">
         <v>23</v>
       </c>
       <c r="D48" s="6" t="s">
@@ -2661,18 +2681,18 @@
       <c r="I48" t="s">
         <v>14</v>
       </c>
-      <c r="J48" t="s">
+      <c r="J48" s="30" t="s">
         <v>111</v>
       </c>
     </row>
     <row r="49" spans="1:10" ht="16" x14ac:dyDescent="0.2">
-      <c r="A49" s="13" t="s">
+      <c r="A49" s="12" t="s">
         <v>44</v>
       </c>
       <c r="B49" t="s">
         <v>109</v>
       </c>
-      <c r="C49" s="17" t="s">
+      <c r="C49" s="16" t="s">
         <v>23</v>
       </c>
       <c r="D49" s="6" t="s">
@@ -2693,18 +2713,18 @@
       <c r="I49" t="s">
         <v>20</v>
       </c>
-      <c r="J49" t="s">
+      <c r="J49" s="30" t="s">
         <v>112</v>
       </c>
     </row>
     <row r="50" spans="1:10" ht="16" x14ac:dyDescent="0.2">
-      <c r="A50" s="13" t="s">
+      <c r="A50" s="12" t="s">
         <v>44</v>
       </c>
       <c r="B50" t="s">
         <v>113</v>
       </c>
-      <c r="C50" s="17" t="s">
+      <c r="C50" s="16" t="s">
         <v>23</v>
       </c>
       <c r="D50" s="6" t="s">
@@ -2725,18 +2745,18 @@
       <c r="I50" t="s">
         <v>14</v>
       </c>
-      <c r="J50" t="s">
+      <c r="J50" s="30" t="s">
         <v>114</v>
       </c>
     </row>
     <row r="51" spans="1:10" ht="16" x14ac:dyDescent="0.2">
-      <c r="A51" s="13" t="s">
+      <c r="A51" s="12" t="s">
         <v>44</v>
       </c>
       <c r="B51" t="s">
         <v>113</v>
       </c>
-      <c r="C51" s="17" t="s">
+      <c r="C51" s="16" t="s">
         <v>23</v>
       </c>
       <c r="D51" s="6" t="s">
@@ -2757,18 +2777,18 @@
       <c r="I51" t="s">
         <v>20</v>
       </c>
-      <c r="J51" t="s">
+      <c r="J51" s="30" t="s">
         <v>115</v>
       </c>
     </row>
     <row r="52" spans="1:10" ht="16" x14ac:dyDescent="0.2">
-      <c r="A52" s="13" t="s">
+      <c r="A52" s="12" t="s">
         <v>44</v>
       </c>
       <c r="B52" t="s">
         <v>116</v>
       </c>
-      <c r="C52" s="17" t="s">
+      <c r="C52" s="16" t="s">
         <v>23</v>
       </c>
       <c r="D52" s="6" t="s">
@@ -2789,18 +2809,18 @@
       <c r="I52" t="s">
         <v>20</v>
       </c>
-      <c r="J52" t="s">
+      <c r="J52" s="30" t="s">
         <v>117</v>
       </c>
     </row>
     <row r="53" spans="1:10" ht="16" x14ac:dyDescent="0.2">
-      <c r="A53" s="13" t="s">
+      <c r="A53" s="12" t="s">
         <v>44</v>
       </c>
       <c r="B53" t="s">
         <v>116</v>
       </c>
-      <c r="C53" s="17" t="s">
+      <c r="C53" s="16" t="s">
         <v>23</v>
       </c>
       <c r="D53" s="6" t="s">
@@ -2821,18 +2841,18 @@
       <c r="I53" t="s">
         <v>20</v>
       </c>
-      <c r="J53" t="s">
+      <c r="J53" s="30" t="s">
         <v>118</v>
       </c>
     </row>
     <row r="54" spans="1:10" ht="16" x14ac:dyDescent="0.2">
-      <c r="A54" s="13" t="s">
+      <c r="A54" s="12" t="s">
         <v>44</v>
       </c>
       <c r="B54" t="s">
         <v>116</v>
       </c>
-      <c r="C54" s="17" t="s">
+      <c r="C54" s="16" t="s">
         <v>23</v>
       </c>
       <c r="D54" s="6" t="s">
@@ -2853,18 +2873,18 @@
       <c r="I54" t="s">
         <v>6</v>
       </c>
-      <c r="J54" t="s">
+      <c r="J54" s="30" t="s">
         <v>119</v>
       </c>
     </row>
     <row r="55" spans="1:10" ht="16" x14ac:dyDescent="0.2">
-      <c r="A55" s="13" t="s">
+      <c r="A55" s="12" t="s">
         <v>44</v>
       </c>
       <c r="B55" t="s">
         <v>116</v>
       </c>
-      <c r="C55" s="17" t="s">
+      <c r="C55" s="16" t="s">
         <v>23</v>
       </c>
       <c r="D55" s="6" t="s">
@@ -2885,18 +2905,18 @@
       <c r="I55" t="s">
         <v>6</v>
       </c>
-      <c r="J55" t="s">
+      <c r="J55" s="30" t="s">
         <v>120</v>
       </c>
     </row>
     <row r="56" spans="1:10" ht="16" x14ac:dyDescent="0.2">
-      <c r="A56" s="13" t="s">
+      <c r="A56" s="12" t="s">
         <v>44</v>
       </c>
       <c r="B56" t="s">
         <v>116</v>
       </c>
-      <c r="C56" s="17" t="s">
+      <c r="C56" s="16" t="s">
         <v>23</v>
       </c>
       <c r="D56" s="6" t="s">
@@ -2917,18 +2937,18 @@
       <c r="I56" t="s">
         <v>6</v>
       </c>
-      <c r="J56" t="s">
+      <c r="J56" s="30" t="s">
         <v>121</v>
       </c>
     </row>
     <row r="57" spans="1:10" ht="16" x14ac:dyDescent="0.2">
-      <c r="A57" s="13" t="s">
+      <c r="A57" s="12" t="s">
         <v>44</v>
       </c>
       <c r="B57" t="s">
         <v>122</v>
       </c>
-      <c r="C57" s="17" t="s">
+      <c r="C57" s="16" t="s">
         <v>23</v>
       </c>
       <c r="D57" s="6" t="s">
@@ -2949,18 +2969,18 @@
       <c r="I57" t="s">
         <v>14</v>
       </c>
-      <c r="J57" t="s">
+      <c r="J57" s="30" t="s">
         <v>123</v>
       </c>
     </row>
     <row r="58" spans="1:10" ht="16" x14ac:dyDescent="0.2">
-      <c r="A58" s="13" t="s">
+      <c r="A58" s="12" t="s">
         <v>44</v>
       </c>
       <c r="B58" t="s">
         <v>124</v>
       </c>
-      <c r="C58" s="17" t="s">
+      <c r="C58" s="16" t="s">
         <v>23</v>
       </c>
       <c r="D58" s="6" t="s">
@@ -2981,18 +3001,18 @@
       <c r="I58" t="s">
         <v>14</v>
       </c>
-      <c r="J58" t="s">
+      <c r="J58" s="30" t="s">
         <v>125</v>
       </c>
     </row>
     <row r="59" spans="1:10" ht="16" x14ac:dyDescent="0.2">
-      <c r="A59" s="13" t="s">
+      <c r="A59" s="12" t="s">
         <v>44</v>
       </c>
       <c r="B59" t="s">
         <v>126</v>
       </c>
-      <c r="C59" s="17" t="s">
+      <c r="C59" s="16" t="s">
         <v>23</v>
       </c>
       <c r="D59" s="6" t="s">
@@ -3013,18 +3033,18 @@
       <c r="I59" t="s">
         <v>95</v>
       </c>
-      <c r="J59" t="s">
+      <c r="J59" s="30" t="s">
         <v>129</v>
       </c>
     </row>
     <row r="60" spans="1:10" ht="16" x14ac:dyDescent="0.2">
-      <c r="A60" s="13" t="s">
+      <c r="A60" s="12" t="s">
         <v>44</v>
       </c>
       <c r="B60" t="s">
         <v>130</v>
       </c>
-      <c r="C60" s="17" t="s">
+      <c r="C60" s="16" t="s">
         <v>23</v>
       </c>
       <c r="D60" s="6" t="s">
@@ -3045,18 +3065,18 @@
       <c r="I60" t="s">
         <v>20</v>
       </c>
-      <c r="J60" t="s">
+      <c r="J60" s="30" t="s">
         <v>131</v>
       </c>
     </row>
     <row r="61" spans="1:10" ht="16" x14ac:dyDescent="0.2">
-      <c r="A61" s="13" t="s">
+      <c r="A61" s="12" t="s">
         <v>44</v>
       </c>
       <c r="B61" t="s">
         <v>130</v>
       </c>
-      <c r="C61" s="17" t="s">
+      <c r="C61" s="16" t="s">
         <v>23</v>
       </c>
       <c r="D61" s="6" t="s">
@@ -3077,18 +3097,18 @@
       <c r="I61" t="s">
         <v>20</v>
       </c>
-      <c r="J61" t="s">
+      <c r="J61" s="30" t="s">
         <v>132</v>
       </c>
     </row>
     <row r="62" spans="1:10" ht="16" x14ac:dyDescent="0.2">
-      <c r="A62" s="13" t="s">
+      <c r="A62" s="12" t="s">
         <v>44</v>
       </c>
       <c r="B62" t="s">
         <v>130</v>
       </c>
-      <c r="C62" s="17" t="s">
+      <c r="C62" s="16" t="s">
         <v>23</v>
       </c>
       <c r="D62" s="6" t="s">
@@ -3109,18 +3129,18 @@
       <c r="I62" t="s">
         <v>20</v>
       </c>
-      <c r="J62" t="s">
+      <c r="J62" s="30" t="s">
         <v>133</v>
       </c>
     </row>
     <row r="63" spans="1:10" ht="16" x14ac:dyDescent="0.2">
-      <c r="A63" s="13" t="s">
+      <c r="A63" s="12" t="s">
         <v>44</v>
       </c>
       <c r="B63" t="s">
         <v>130</v>
       </c>
-      <c r="C63" s="17" t="s">
+      <c r="C63" s="16" t="s">
         <v>23</v>
       </c>
       <c r="D63" s="6" t="s">
@@ -3141,18 +3161,18 @@
       <c r="I63" t="s">
         <v>12</v>
       </c>
-      <c r="J63" t="s">
+      <c r="J63" s="30" t="s">
         <v>136</v>
       </c>
     </row>
     <row r="64" spans="1:10" ht="16" x14ac:dyDescent="0.2">
-      <c r="A64" s="13" t="s">
+      <c r="A64" s="12" t="s">
         <v>44</v>
       </c>
       <c r="B64" t="s">
         <v>137</v>
       </c>
-      <c r="C64" s="17" t="s">
+      <c r="C64" s="16" t="s">
         <v>23</v>
       </c>
       <c r="D64" s="6" t="s">
@@ -3173,18 +3193,18 @@
       <c r="I64" t="s">
         <v>20</v>
       </c>
-      <c r="J64" t="s">
+      <c r="J64" s="30" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="65" spans="1:10" ht="16" x14ac:dyDescent="0.2">
-      <c r="A65" s="13" t="s">
+    <row r="65" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+      <c r="A65" s="12" t="s">
         <v>44</v>
       </c>
       <c r="B65" t="s">
         <v>138</v>
       </c>
-      <c r="C65" s="17" t="s">
+      <c r="C65" s="16" t="s">
         <v>23</v>
       </c>
       <c r="D65" s="6" t="s">
@@ -3205,18 +3225,18 @@
       <c r="I65" t="s">
         <v>14</v>
       </c>
-      <c r="J65" t="s">
+      <c r="J65" s="30" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="66" spans="1:10" ht="16" x14ac:dyDescent="0.2">
-      <c r="A66" s="13" t="s">
+    <row r="66" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+      <c r="A66" s="12" t="s">
         <v>44</v>
       </c>
       <c r="B66" t="s">
         <v>141</v>
       </c>
-      <c r="C66" s="17" t="s">
+      <c r="C66" s="16" t="s">
         <v>23</v>
       </c>
       <c r="D66" s="6" t="s">
@@ -3237,18 +3257,18 @@
       <c r="I66" t="s">
         <v>20</v>
       </c>
-      <c r="J66" t="s">
+      <c r="J66" s="30" t="s">
         <v>142</v>
       </c>
     </row>
-    <row r="67" spans="1:10" ht="16" x14ac:dyDescent="0.2">
-      <c r="A67" s="13" t="s">
+    <row r="67" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+      <c r="A67" s="12" t="s">
         <v>44</v>
       </c>
       <c r="B67" t="s">
         <v>141</v>
       </c>
-      <c r="C67" s="17" t="s">
+      <c r="C67" s="16" t="s">
         <v>23</v>
       </c>
       <c r="D67" s="6" t="s">
@@ -3269,18 +3289,18 @@
       <c r="I67" t="s">
         <v>20</v>
       </c>
-      <c r="J67" t="s">
+      <c r="J67" s="30" t="s">
         <v>143</v>
       </c>
     </row>
-    <row r="68" spans="1:10" ht="16" x14ac:dyDescent="0.2">
-      <c r="A68" s="13" t="s">
+    <row r="68" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+      <c r="A68" s="12" t="s">
         <v>44</v>
       </c>
       <c r="B68" t="s">
         <v>144</v>
       </c>
-      <c r="C68" s="17" t="s">
+      <c r="C68" s="16" t="s">
         <v>23</v>
       </c>
       <c r="D68" s="6" t="s">
@@ -3301,18 +3321,18 @@
       <c r="I68" t="s">
         <v>6</v>
       </c>
-      <c r="J68" t="s">
+      <c r="J68" s="30" t="s">
         <v>145</v>
       </c>
     </row>
-    <row r="69" spans="1:10" ht="16" x14ac:dyDescent="0.2">
-      <c r="A69" s="13" t="s">
+    <row r="69" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+      <c r="A69" s="12" t="s">
         <v>44</v>
       </c>
       <c r="B69" t="s">
         <v>144</v>
       </c>
-      <c r="C69" s="17" t="s">
+      <c r="C69" s="16" t="s">
         <v>23</v>
       </c>
       <c r="D69" s="6" t="s">
@@ -3333,18 +3353,18 @@
       <c r="I69" t="s">
         <v>6</v>
       </c>
-      <c r="J69" t="s">
+      <c r="J69" s="30" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="70" spans="1:10" ht="16" x14ac:dyDescent="0.2">
-      <c r="A70" s="13" t="s">
+    <row r="70" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+      <c r="A70" s="12" t="s">
         <v>44</v>
       </c>
       <c r="B70" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="C70" s="14" t="s">
+      <c r="C70" s="13" t="s">
         <v>17</v>
       </c>
       <c r="D70" s="6" t="s">
@@ -3362,21 +3382,21 @@
       <c r="H70" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="I70" s="11" t="s">
+      <c r="I70" s="27" t="s">
         <v>20</v>
       </c>
-      <c r="J70" s="12" t="s">
+      <c r="J70" s="11" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="71" spans="1:10" ht="16" x14ac:dyDescent="0.2">
-      <c r="A71" s="13" t="s">
+    <row r="71" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+      <c r="A71" s="12" t="s">
         <v>44</v>
       </c>
       <c r="B71" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="C71" s="15" t="s">
+      <c r="C71" s="14" t="s">
         <v>47</v>
       </c>
       <c r="D71" s="6" t="s">
@@ -3394,63 +3414,77 @@
       <c r="H71" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="I71" s="11" t="s">
+      <c r="I71" s="27" t="s">
         <v>20</v>
       </c>
-      <c r="J71" s="12" t="s">
+      <c r="J71" s="11" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="72" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A72" s="13"/>
-      <c r="B72" s="8"/>
-      <c r="C72" s="8"/>
-      <c r="D72" s="6"/>
-      <c r="E72" s="7"/>
-      <c r="F72" s="10"/>
-      <c r="G72" s="8"/>
-      <c r="H72" s="8"/>
-      <c r="I72" s="11"/>
-      <c r="J72" s="12"/>
-    </row>
-    <row r="73" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A73" s="13"/>
-      <c r="B73" s="8"/>
-      <c r="C73" s="8"/>
-      <c r="D73" s="6"/>
-      <c r="E73" s="7"/>
-      <c r="F73" s="10"/>
-      <c r="G73" s="8"/>
-      <c r="H73" s="8"/>
-      <c r="I73" s="11"/>
-      <c r="J73" s="12"/>
-    </row>
-    <row r="74" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A74" s="13"/>
-      <c r="B74" s="8"/>
-      <c r="C74" s="8"/>
-      <c r="D74" s="6"/>
-      <c r="E74" s="7"/>
-      <c r="F74" s="10"/>
-      <c r="G74" s="8"/>
-      <c r="H74" s="8"/>
-      <c r="I74" s="11"/>
-      <c r="J74" s="12"/>
-    </row>
-    <row r="75" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A75" s="13"/>
-      <c r="B75" s="8"/>
-      <c r="C75" s="8"/>
-      <c r="D75" s="6"/>
-      <c r="E75" s="7"/>
-      <c r="F75" s="10"/>
-      <c r="G75" s="8"/>
-      <c r="H75" s="8"/>
-      <c r="I75" s="11"/>
-      <c r="J75" s="12"/>
-    </row>
-    <row r="76" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="J76" s="12"/>
+    <row r="72" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A72"/>
+      <c r="B72"/>
+      <c r="C72"/>
+      <c r="D72"/>
+      <c r="E72"/>
+      <c r="F72"/>
+      <c r="G72"/>
+      <c r="H72"/>
+      <c r="I72"/>
+      <c r="J72"/>
+      <c r="K72"/>
+    </row>
+    <row r="73" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A73"/>
+      <c r="B73"/>
+      <c r="C73"/>
+      <c r="D73"/>
+      <c r="E73"/>
+      <c r="F73"/>
+      <c r="G73"/>
+      <c r="H73"/>
+      <c r="I73"/>
+      <c r="J73"/>
+      <c r="K73"/>
+    </row>
+    <row r="74" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A74"/>
+      <c r="B74"/>
+      <c r="C74"/>
+      <c r="D74"/>
+      <c r="E74"/>
+      <c r="F74"/>
+      <c r="G74"/>
+      <c r="H74"/>
+      <c r="I74"/>
+      <c r="J74"/>
+      <c r="K74"/>
+    </row>
+    <row r="75" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A75"/>
+      <c r="B75"/>
+      <c r="C75"/>
+      <c r="D75"/>
+      <c r="E75"/>
+      <c r="F75"/>
+      <c r="G75"/>
+      <c r="H75"/>
+      <c r="I75"/>
+      <c r="J75"/>
+      <c r="K75"/>
+    </row>
+    <row r="76" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A76"/>
+      <c r="B76"/>
+      <c r="C76"/>
+      <c r="D76"/>
+      <c r="E76"/>
+      <c r="F76"/>
+      <c r="G76"/>
+      <c r="H76"/>
+      <c r="I76"/>
+      <c r="J76"/>
+      <c r="K76"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -3474,6 +3508,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="acff8847-a8fa-457e-8010-fe71e962d383">
@@ -3482,15 +3525,6 @@
     <TaxCatchAll xmlns="94c72131-11e1-48b9-8020-84fe1105e8cb" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3755,20 +3789,20 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9F1695B6-E3F5-4F5D-B7E5-3E0452B0E8F0}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{35538F82-A7FF-48A8-93E6-6CDB157BBBDB}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
     <ds:schemaRef ds:uri="acff8847-a8fa-457e-8010-fe71e962d383"/>
     <ds:schemaRef ds:uri="94c72131-11e1-48b9-8020-84fe1105e8cb"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9F1695B6-E3F5-4F5D-B7E5-3E0452B0E8F0}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>